<commit_message>
Improve season, player, and lineup workflows
</commit_message>
<xml_diff>
--- a/assets/AlphaOpen_Season_Reload_Template.xlsx
+++ b/assets/AlphaOpen_Season_Reload_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R1c6d42911f144ab1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season" sheetId="2" r:id="R1b21c6ce2da54cb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Captains" sheetId="3" r:id="Raf8d5f4c83ee4dfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Roster" sheetId="4" r:id="R2385bbda66fa4e76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Schedule" sheetId="5" r:id="Rdf223f1d4eef4168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R8615858c6d6d458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season" sheetId="2" r:id="Rc4152165fbc84792"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Captains" sheetId="3" r:id="R78a1814868d64da5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Roster" sheetId="4" r:id="R3eca6fae996f4c30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Schedule" sheetId="5" r:id="R18657884e3ea482c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -363,7 +363,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>AlphaOpen Season Reload Template</x:v>
+        <x:v>AlphaOpen New Season Upload Template</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -373,7 +373,7 @@
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Use this workbook after Reset Season Data. Do not rename the four required data tabs or their headers.</x:v>
+        <x:v>Use this workbook to upload a new season. Do not rename the four required data tabs or their headers.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -408,10 +408,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
-        <x:v>Enter eight teams and captains.</x:v>
+        <x:v>Enter the season roster using existing Player IDs and emails.</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
-        <x:v>Captain Player ID and email must match Player Master.</x:v>
+        <x:v>Each player must already exist in the application; IDs and emails must match.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -463,15 +463,15 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
-        <x:v>Run Identity Reconciliation after upload.</x:v>
+        <x:v>Review the validation results and correct every error.</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
-        <x:v>Confirms Player ID/name and public/private parity.</x:v>
+        <x:v>The upload is not committed until the confirmation step succeeds.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>Important: Season Master, Player Master, Venue Master and global User records are retained by reset. Season memberships, teams, rosters, schedules, lineups, scores and published data are rebuilt.</x:v>
+        <x:v>This upload includes only Season, Captains, Team Roster and Weekly Schedule. Lineup Approver assignments, venues and Player Master are managed separately in the application.</x:v>
       </x:c>
       <x:c r="B14" s="14"/>
       <x:c r="C14" s="14"/>

</xml_diff>